<commit_message>
uradjen ios dobavljaca i avansa
</commit_message>
<xml_diff>
--- a/pomocna_knjiga_avansa_excel.xlsx
+++ b/pomocna_knjiga_avansa_excel.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
-    <t>PLAĆENI AVANSI OD 01.01.2024. - 22.11.2024.</t>
+    <t>PLAĆENI AVANSI OD 01.01.2025. - 30.11.2025.</t>
   </si>
   <si>
     <t>Početno</t>
@@ -40,19 +40,13 @@
     <t>Potražuje</t>
   </si>
   <si>
-    <t xml:space="preserve"> OFFICE&amp;MORE</t>
-  </si>
-  <si>
     <t>AMSS</t>
   </si>
   <si>
-    <t>CHILL OUT</t>
-  </si>
-  <si>
-    <t>HTUP PARK</t>
-  </si>
-  <si>
-    <t>METRO</t>
+    <t>BC GROUP</t>
+  </si>
+  <si>
+    <t>JKP PARKING SERVIS</t>
   </si>
   <si>
     <t>NIS GASPROM</t>
@@ -61,7 +55,13 @@
     <t>PTT POŠTA</t>
   </si>
   <si>
+    <t>SAS CS COMPANY</t>
+  </si>
+  <si>
     <t>SEMINARI SRBIJE</t>
+  </si>
+  <si>
+    <t>SRBOLAB</t>
   </si>
 </sst>
 </file>
@@ -421,9 +421,11 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -493,22 +495,22 @@
         <v>8</v>
       </c>
       <c r="B4" s="3">
-        <v>17598.8</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3">
         <v>0</v>
       </c>
       <c r="D4" s="3">
-        <v>0</v>
+        <v>28200.00</v>
       </c>
       <c r="E4" s="3">
-        <v>17598.8</v>
+        <v>28200.00</v>
       </c>
       <c r="F4" s="3">
-        <v>17598.8</v>
+        <v>28200.00</v>
       </c>
       <c r="G4" s="3">
-        <v>17598.8</v>
+        <v>28200.00</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
@@ -528,16 +530,16 @@
         <v>0</v>
       </c>
       <c r="D5" s="3">
-        <v>9400</v>
+        <v>49979.00</v>
       </c>
       <c r="E5" s="3">
-        <v>9400</v>
+        <v>49979.00</v>
       </c>
       <c r="F5" s="3">
-        <v>9400</v>
+        <v>49979.00</v>
       </c>
       <c r="G5" s="3">
-        <v>9400</v>
+        <v>49979.00</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
@@ -551,25 +553,25 @@
         <v>10</v>
       </c>
       <c r="B6" s="3">
-        <v>12000</v>
+        <v>323238.00</v>
       </c>
       <c r="C6" s="3">
         <v>0</v>
       </c>
       <c r="D6" s="3">
-        <v>0</v>
+        <v>265947.82</v>
       </c>
       <c r="E6" s="3">
-        <v>0</v>
+        <v>266640.82</v>
       </c>
       <c r="F6" s="3">
-        <v>12000</v>
+        <v>589185.82</v>
       </c>
       <c r="G6" s="3">
-        <v>0</v>
+        <v>266640.82</v>
       </c>
       <c r="H6" s="3">
-        <v>12000</v>
+        <v>322545.00</v>
       </c>
       <c r="I6" s="3">
         <v>0</v>
@@ -580,25 +582,25 @@
         <v>11</v>
       </c>
       <c r="B7" s="3">
-        <v>8875</v>
+        <v>86411.69</v>
       </c>
       <c r="C7" s="3">
         <v>0</v>
       </c>
       <c r="D7" s="3">
-        <v>0</v>
+        <v>189800.00</v>
       </c>
       <c r="E7" s="3">
-        <v>0</v>
+        <v>227277.37</v>
       </c>
       <c r="F7" s="3">
-        <v>8875</v>
+        <v>276211.69</v>
       </c>
       <c r="G7" s="3">
-        <v>0</v>
+        <v>227277.37</v>
       </c>
       <c r="H7" s="3">
-        <v>8875</v>
+        <v>48934.32</v>
       </c>
       <c r="I7" s="3">
         <v>0</v>
@@ -609,25 +611,25 @@
         <v>12</v>
       </c>
       <c r="B8" s="3">
-        <v>486.54</v>
+        <v>1207917.49</v>
       </c>
       <c r="C8" s="3">
         <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>0</v>
+        <v>15000.00</v>
       </c>
       <c r="E8" s="3">
-        <v>0</v>
+        <v>505199.00</v>
       </c>
       <c r="F8" s="3">
-        <v>486.54</v>
+        <v>1222917.49</v>
       </c>
       <c r="G8" s="3">
-        <v>0</v>
+        <v>505199.00</v>
       </c>
       <c r="H8" s="3">
-        <v>486.54</v>
+        <v>717718.49</v>
       </c>
       <c r="I8" s="3">
         <v>0</v>
@@ -638,25 +640,25 @@
         <v>13</v>
       </c>
       <c r="B9" s="3">
-        <v>277137.68</v>
+        <v>0</v>
       </c>
       <c r="C9" s="3">
         <v>0</v>
       </c>
       <c r="D9" s="3">
-        <v>76048.8</v>
+        <v>224160.00</v>
       </c>
       <c r="E9" s="3">
-        <v>219780.48</v>
+        <v>224160.00</v>
       </c>
       <c r="F9" s="3">
-        <v>353186.48</v>
+        <v>224160.00</v>
       </c>
       <c r="G9" s="3">
-        <v>219780.48</v>
+        <v>224160.00</v>
       </c>
       <c r="H9" s="3">
-        <v>133406</v>
+        <v>0</v>
       </c>
       <c r="I9" s="3">
         <v>0</v>
@@ -667,25 +669,25 @@
         <v>14</v>
       </c>
       <c r="B10" s="3">
-        <v>397003.49</v>
+        <v>68880.00</v>
       </c>
       <c r="C10" s="3">
         <v>0</v>
       </c>
       <c r="D10" s="3">
-        <v>400000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="3">
-        <v>590523</v>
+        <v>51600.00</v>
       </c>
       <c r="F10" s="3">
-        <v>797003.49</v>
+        <v>68880.00</v>
       </c>
       <c r="G10" s="3">
-        <v>590523</v>
+        <v>51600.00</v>
       </c>
       <c r="H10" s="3">
-        <v>206480.49</v>
+        <v>17280.00</v>
       </c>
       <c r="I10" s="3">
         <v>0</v>
@@ -696,25 +698,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="3">
-        <v>68880</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3">
         <v>0</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>10000.00</v>
       </c>
       <c r="E11" s="3">
-        <v>0</v>
+        <v>10000.00</v>
       </c>
       <c r="F11" s="3">
-        <v>68880</v>
+        <v>10000.00</v>
       </c>
       <c r="G11" s="3">
-        <v>0</v>
+        <v>10000.00</v>
       </c>
       <c r="H11" s="3">
-        <v>68880</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3">
         <v>0</v>

</xml_diff>